<commit_message>
add a report for IA profiles
</commit_message>
<xml_diff>
--- a/public/templates/PERSONNAL_LOCATOR_SLIP.xlsx
+++ b/public/templates/PERSONNAL_LOCATOR_SLIP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\AIMS\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F204EDF2-DD2D-4991-BF1D-03331A8A5496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007EC087-CDD6-4B8F-AF66-A17D17E2D852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C94C062E-6212-4E28-A84B-528FAA87AA11}"/>
   </bookViews>
@@ -273,7 +273,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -314,9 +314,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -347,6 +344,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -359,10 +359,13 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1977,15 +1980,15 @@
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E3" s="30" t="s">
+      <c r="E3" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="E4" s="3" t="s">
@@ -2010,8 +2013,8 @@
       <c r="K6" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="L6" s="31"/>
-      <c r="M6" s="31"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="4"/>
@@ -2055,16 +2058,16 @@
       <c r="L9" s="4"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="32"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
       <c r="J10" s="6" t="s">
         <v>7</v>
       </c>
@@ -2084,24 +2087,24 @@
       <c r="G11" s="33"/>
       <c r="H11" s="33"/>
       <c r="I11" s="33"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="32"/>
-      <c r="L11" s="32"/>
-      <c r="M11" s="32"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="25"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="24"/>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="4"/>
@@ -2184,11 +2187,11 @@
       <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
-      <c r="I18" s="31"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="31"/>
-      <c r="L18" s="31"/>
-      <c r="M18" s="31"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
+      <c r="K18" s="30"/>
+      <c r="L18" s="30"/>
+      <c r="M18" s="30"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B19" s="4"/>
@@ -2198,13 +2201,13 @@
       <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="15"/>
-      <c r="I19" s="37" t="s">
+      <c r="I19" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="J19" s="37"/>
-      <c r="K19" s="37"/>
-      <c r="L19" s="37"/>
-      <c r="M19" s="37"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="32"/>
+      <c r="L19" s="32"/>
+      <c r="M19" s="32"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D20" s="21" t="s">
@@ -2227,18 +2230,20 @@
       <c r="M22" s="36"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
+      <c r="B23" s="39"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="39"/>
+      <c r="E23" s="39"/>
+      <c r="F23" s="39"/>
+      <c r="G23" s="39"/>
       <c r="H23" s="15"/>
-      <c r="I23" s="23" t="s">
+      <c r="I23" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="23"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
     </row>
     <row r="24" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="13"/>
@@ -2282,47 +2287,47 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B27" s="28" t="s">
+      <c r="B27" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
-      <c r="G27" s="26"/>
+      <c r="C27" s="27"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
+      <c r="F28" s="28"/>
+      <c r="G28" s="28"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="27"/>
-      <c r="K30" s="27"/>
-      <c r="L30" s="27"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="27"/>
-      <c r="L31" s="27"/>
+      <c r="B31" s="26"/>
+      <c r="C31" s="26"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="26"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="26"/>
+      <c r="I31" s="26"/>
+      <c r="J31" s="26"/>
+      <c r="K31" s="26"/>
+      <c r="L31" s="26"/>
     </row>
     <row r="36" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="17"/>
@@ -2359,15 +2364,15 @@
       <c r="J39" s="1"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="E40" s="30" t="s">
+      <c r="E40" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="F40" s="30"/>
-      <c r="G40" s="30"/>
-      <c r="H40" s="30"/>
-      <c r="I40" s="30"/>
-      <c r="J40" s="30"/>
-      <c r="K40" s="30"/>
+      <c r="F40" s="29"/>
+      <c r="G40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="29"/>
+      <c r="K40" s="29"/>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="E41" s="3" t="s">
@@ -2392,11 +2397,11 @@
       <c r="K43" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="L43" s="31">
+      <c r="L43" s="30">
         <f>L6</f>
         <v>0</v>
       </c>
-      <c r="M43" s="31"/>
+      <c r="M43" s="30"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B44" s="4"/>
@@ -2440,19 +2445,19 @@
       <c r="L46" s="4"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B47" s="24" t="s">
+      <c r="B47" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="24"/>
-      <c r="D47" s="24"/>
-      <c r="E47" s="24"/>
-      <c r="F47" s="24"/>
-      <c r="G47" s="24"/>
-      <c r="H47" s="32">
+      <c r="C47" s="23"/>
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="31">
         <f>H10</f>
         <v>0</v>
       </c>
-      <c r="I47" s="32"/>
+      <c r="I47" s="31"/>
       <c r="J47" s="6" t="s">
         <v>7</v>
       </c>
@@ -2475,27 +2480,27 @@
       <c r="G48" s="33"/>
       <c r="H48" s="33"/>
       <c r="I48" s="33"/>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="32"/>
+      <c r="J48" s="31"/>
+      <c r="K48" s="31"/>
+      <c r="L48" s="31"/>
+      <c r="M48" s="31"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B49" s="25">
+      <c r="B49" s="24">
         <f>B12</f>
         <v>0</v>
       </c>
-      <c r="C49" s="25"/>
-      <c r="D49" s="25"/>
-      <c r="E49" s="25"/>
-      <c r="F49" s="25"/>
-      <c r="G49" s="25"/>
-      <c r="H49" s="25"/>
-      <c r="I49" s="25"/>
-      <c r="J49" s="25"/>
-      <c r="K49" s="25"/>
-      <c r="L49" s="25"/>
-      <c r="M49" s="25"/>
+      <c r="C49" s="24"/>
+      <c r="D49" s="24"/>
+      <c r="E49" s="24"/>
+      <c r="F49" s="24"/>
+      <c r="G49" s="24"/>
+      <c r="H49" s="24"/>
+      <c r="I49" s="24"/>
+      <c r="J49" s="24"/>
+      <c r="K49" s="24"/>
+      <c r="L49" s="24"/>
+      <c r="M49" s="24"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
@@ -2587,14 +2592,14 @@
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
-      <c r="I55" s="31">
+      <c r="I55" s="30">
         <f>I18</f>
         <v>0</v>
       </c>
-      <c r="J55" s="31"/>
-      <c r="K55" s="31"/>
-      <c r="L55" s="31"/>
-      <c r="M55" s="31"/>
+      <c r="J55" s="30"/>
+      <c r="K55" s="30"/>
+      <c r="L55" s="30"/>
+      <c r="M55" s="30"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B56" s="4"/>
@@ -2604,13 +2609,13 @@
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="15"/>
-      <c r="I56" s="37" t="s">
+      <c r="I56" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="J56" s="37"/>
-      <c r="K56" s="37"/>
-      <c r="L56" s="37"/>
-      <c r="M56" s="37"/>
+      <c r="J56" s="32"/>
+      <c r="K56" s="32"/>
+      <c r="L56" s="32"/>
+      <c r="M56" s="32"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="D57" s="21" t="s">
@@ -2636,21 +2641,23 @@
       <c r="M59" s="36"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C60" s="22">
-        <f>C23</f>
+      <c r="B60" s="37">
+        <f>B23</f>
         <v>0</v>
       </c>
-      <c r="D60" s="22"/>
-      <c r="E60" s="22"/>
-      <c r="F60" s="22"/>
+      <c r="C60" s="37"/>
+      <c r="D60" s="37"/>
+      <c r="E60" s="37"/>
+      <c r="F60" s="37"/>
+      <c r="G60" s="37"/>
       <c r="H60" s="15"/>
-      <c r="I60" s="23" t="s">
+      <c r="I60" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="J60" s="23"/>
-      <c r="K60" s="23"/>
-      <c r="L60" s="23"/>
-      <c r="M60" s="23"/>
+      <c r="J60" s="22"/>
+      <c r="K60" s="22"/>
+      <c r="L60" s="22"/>
+      <c r="M60" s="22"/>
     </row>
     <row r="61" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="13"/>
@@ -2694,51 +2701,50 @@
       </c>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B64" s="28" t="s">
+      <c r="B64" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C64" s="28"/>
-      <c r="D64" s="28"/>
-      <c r="E64" s="26"/>
-      <c r="F64" s="26"/>
-      <c r="G64" s="26"/>
+      <c r="C64" s="27"/>
+      <c r="D64" s="27"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="25"/>
+      <c r="G64" s="25"/>
     </row>
     <row r="65" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="E65" s="23" t="s">
+      <c r="E65" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="F65" s="29"/>
-      <c r="G65" s="29"/>
+      <c r="F65" s="28"/>
+      <c r="G65" s="28"/>
     </row>
     <row r="66" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B66" s="27"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="27"/>
-      <c r="E66" s="27"/>
-      <c r="F66" s="27"/>
-      <c r="G66" s="27"/>
-      <c r="H66" s="27"/>
-      <c r="I66" s="27"/>
-      <c r="J66" s="27"/>
-      <c r="K66" s="27"/>
-      <c r="L66" s="27"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="26"/>
+      <c r="D66" s="26"/>
+      <c r="E66" s="26"/>
+      <c r="F66" s="26"/>
+      <c r="G66" s="26"/>
+      <c r="H66" s="26"/>
+      <c r="I66" s="26"/>
+      <c r="J66" s="26"/>
+      <c r="K66" s="26"/>
+      <c r="L66" s="26"/>
     </row>
     <row r="67" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="27"/>
-      <c r="F67" s="27"/>
-      <c r="G67" s="27"/>
-      <c r="H67" s="27"/>
-      <c r="I67" s="27"/>
-      <c r="J67" s="27"/>
-      <c r="K67" s="27"/>
-      <c r="L67" s="27"/>
+      <c r="B67" s="26"/>
+      <c r="C67" s="26"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="26"/>
+      <c r="F67" s="26"/>
+      <c r="G67" s="26"/>
+      <c r="H67" s="26"/>
+      <c r="I67" s="26"/>
+      <c r="J67" s="26"/>
+      <c r="K67" s="26"/>
+      <c r="L67" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C22:F22"/>
     <mergeCell ref="I22:M22"/>
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="E45:K45"/>
@@ -2747,15 +2753,16 @@
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="D16:H16"/>
     <mergeCell ref="I18:M18"/>
+    <mergeCell ref="B23:G23"/>
     <mergeCell ref="I55:M55"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="C59:F59"/>
-    <mergeCell ref="C60:F60"/>
     <mergeCell ref="I59:M59"/>
     <mergeCell ref="I60:M60"/>
     <mergeCell ref="D57:E57"/>
     <mergeCell ref="I56:M56"/>
     <mergeCell ref="D53:H53"/>
+    <mergeCell ref="B60:G60"/>
     <mergeCell ref="B64:D64"/>
     <mergeCell ref="E64:G64"/>
     <mergeCell ref="E65:G65"/>
@@ -2772,7 +2779,6 @@
     <mergeCell ref="E2:I2"/>
     <mergeCell ref="E38:H38"/>
     <mergeCell ref="D20:E20"/>
-    <mergeCell ref="C23:F23"/>
     <mergeCell ref="I23:M23"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="B12:M12"/>
@@ -2785,6 +2791,7 @@
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="I19:M19"/>
+    <mergeCell ref="C22:F22"/>
   </mergeCells>
   <pageMargins left="0.74" right="0.21" top="0.75" bottom="0.75" header="0.34" footer="0.3"/>
   <pageSetup paperSize="14" scale="78" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>